<commit_message>
coverage: add 'Новый контейнер' sheet with live formulas
Second sheet in the brand-sorted coverage workbook: 41 low-stock SKUs
(<150 days, FarmStay excluded). Formulas: order = target_months × 2-store
demand − current total; weight = qty × kg/unit. Parameter cells (transit,
target months, store multiplier, kg/unit, 26t/120k caps) drive recompute.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XzNBEf4vaaEHRqeR8ZkfFA
</commit_message>
<xml_diff>
--- a/outputs/coverage/pokrytie_po_brendam_2026-06-30.xlsx
+++ b/outputs/coverage/pokrytie_po_brendam_2026-06-30.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Покрытие" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Новый контейнер" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,8 +33,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00C55A11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +60,11 @@
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C55A11"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -68,13 +78,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5582,7 +5596,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr"/>
       <c r="C126" t="inlineStr">
         <is>
           <t>SKIN1004 Madagascar Centella Ampoule 55ml</t>
@@ -5619,7 +5632,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr"/>
       <c r="C127" t="inlineStr">
         <is>
           <t>Пенка для умыванияCELIMAX THE REAL NONI ACNE BUBBLE CLEANSER</t>
@@ -5656,7 +5668,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr"/>
       <c r="C128" t="inlineStr">
         <is>
           <t>Сыворотка-лифтинг с ПДРН и пептидами Medicube, 30 мл/PDRN PI</t>
@@ -5693,7 +5704,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr"/>
       <c r="C129" t="inlineStr">
         <is>
           <t xml:space="preserve">1025 DOKDO BUBBLE FOAM_150ml (дозатор ) </t>
@@ -5730,7 +5740,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr"/>
       <c r="C130" t="inlineStr">
         <is>
           <t>Блеск Плампер для губ VT REEDLE SHOT LIP PLUMPER EXPERT</t>
@@ -5767,7 +5776,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr"/>
       <c r="C131" t="inlineStr">
         <is>
           <t>Гель для душа от прыщей с кислотами/PINE CALMING CICA BODY W</t>
@@ -5804,7 +5812,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr"/>
       <c r="C132" t="inlineStr">
         <is>
           <t xml:space="preserve">Сыворотка для лица от морщин с микроиглами 7500 и пдрн/PDRN </t>
@@ -5841,7 +5848,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr"/>
       <c r="C133" t="inlineStr">
         <is>
           <t>Осветляющий Крем от пигментации с Транексамовой Кислотой/[De</t>
@@ -5878,7 +5884,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr"/>
       <c r="C134" t="inlineStr">
         <is>
           <t>DEOPROCE SHAMPOO - BLACK GARLIC INTENSME ENERGY [1000ml]</t>
@@ -5915,7 +5920,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr"/>
       <c r="C135" t="inlineStr">
         <is>
           <t>Увлажняющий тонер-эссенция для лица с аденозином 7500 ppm/Ad</t>
@@ -5952,7 +5956,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr"/>
       <c r="C136" t="inlineStr">
         <is>
           <t xml:space="preserve">CELIMAX DUAL BARRIER MILD GEL CLEANSER 200ML(дозатор) </t>
@@ -5989,7 +5992,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr"/>
       <c r="C137" t="inlineStr">
         <is>
           <t>CELIMAX OIL CONTROL MOISTURIZING CREAM 80ML</t>
@@ -6026,7 +6028,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr"/>
       <c r="C138" t="inlineStr">
         <is>
           <t xml:space="preserve">Сыворотка с пептидами Матриксил 15% от морщин/ </t>
@@ -6063,7 +6064,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr"/>
       <c r="C139" t="inlineStr">
         <is>
           <t>SKIN1004 Madagascar Centella Soothing Cream 75ml</t>
@@ -6100,7 +6100,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr"/>
       <c r="C140" t="inlineStr">
         <is>
           <t>BIFIDA BIOME AMPOULE TONER 210 мл</t>
@@ -6137,7 +6136,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr"/>
       <c r="C141" t="inlineStr">
         <is>
           <t>CELIMAX PORE+DARK SPOT BRIGHTENING KIT</t>
@@ -6174,7 +6172,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr"/>
       <c r="C142" t="inlineStr">
         <is>
           <t>Тонер  для лица увлажняющий от прыщей Корея/EXOSOME CICA TON</t>
@@ -6211,7 +6208,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr"/>
       <c r="C143" t="inlineStr">
         <is>
           <t>CELIMAX THE REAL NONI REFRESH CLAY MASK 120G</t>
@@ -6248,7 +6244,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr"/>
       <c r="C144" t="inlineStr">
         <is>
           <t>CELIMAX THE REAL NONI CALMING GLOW PAD 50PADS,</t>
@@ -6285,7 +6280,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr"/>
       <c r="C145" t="inlineStr">
         <is>
           <t>VT REEDLE SHOT LIFTING EYE CREAM</t>
@@ -6322,7 +6316,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr"/>
       <c r="C146" t="inlineStr">
         <is>
           <t>CELIMAX DERMA NATURE GLUTATHIONE LONGLASTING TONE-UP CREAM 3</t>
@@ -6359,7 +6352,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr"/>
       <c r="C147" t="inlineStr">
         <is>
           <t xml:space="preserve">Крем для лица увлажняющий для проблемной кожи с сосной/PINE </t>
@@ -6396,7 +6388,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr"/>
       <c r="C148" t="inlineStr">
         <is>
           <t>DEOPROCE SHAMPOO - ARGAN SILKY MOISTURE</t>
@@ -6433,7 +6424,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr"/>
       <c r="C149" t="inlineStr">
         <is>
           <t>CELIMAX JI WOO GAE CICA BHA ACNE FOAM CLEANSING 150ML</t>
@@ -6470,7 +6460,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr"/>
       <c r="C150" t="inlineStr">
         <is>
           <t>Крем для лица c Бакучиолом и Микроиглами от морщин/ Bakuchio</t>
@@ -6507,7 +6496,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr"/>
       <c r="C151" t="inlineStr">
         <is>
           <t>CELIMAX THE REAL CICA SOOTHING CREAM 50ML</t>
@@ -6544,7 +6532,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr"/>
       <c r="C152" t="inlineStr">
         <is>
           <t>Крем для лица укрепляющий с ретиналем 300ppm/[Derma Factory]</t>
@@ -6581,7 +6568,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr"/>
       <c r="C153" t="inlineStr">
         <is>
           <t>Интенсивная антивозрастная сыворотка для лица PDRN 4%, 30 мл</t>
@@ -6618,7 +6604,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr"/>
       <c r="C154" t="inlineStr">
         <is>
           <t>Сыворотка для лица осветляющая от пигментации/[Derma Factory</t>
@@ -6655,7 +6640,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr"/>
       <c r="C155" t="inlineStr">
         <is>
           <t>CELIMAX DERMA NATURE RELIEF MADECICA PH BALANCING FOAM CLEAN</t>
@@ -6692,7 +6676,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr"/>
       <c r="C156" t="inlineStr">
         <is>
           <t xml:space="preserve">SOYBEAN SERUM_50ml/Сыворотка для лица увлажняющая от морщин </t>
@@ -6729,7 +6712,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr"/>
       <c r="C157" t="inlineStr">
         <is>
           <t>CELIMAX JI WOO GAE ONE STEP MILD CLEANSING PAD 60PADS</t>
@@ -6766,7 +6748,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B158" t="inlineStr"/>
       <c r="C158" t="inlineStr">
         <is>
           <t>ROUND LAB CAMELLIA DEEP COLLAGEN FIRMING CREAM_50ml</t>
@@ -6803,7 +6784,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr"/>
       <c r="C159" t="inlineStr">
         <is>
           <t>CELIMAX OIL CONTROL CAPSULE ESSENCE 30ML</t>
@@ -6840,7 +6820,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B160" t="inlineStr"/>
       <c r="C160" t="inlineStr">
         <is>
           <t>CELIMAX THE REAL CICA NIACINAMIDE AC CALMING SERUM 40ML</t>
@@ -6877,7 +6856,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B161" t="inlineStr"/>
       <c r="C161" t="inlineStr">
         <is>
           <t>Пенка очищающая для лица от прыщей с сосной и кислотами/PINE</t>
@@ -6914,7 +6892,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr"/>
       <c r="C162" t="inlineStr">
         <is>
           <t>1025 DOKDO CREAM_80ml</t>
@@ -6951,7 +6928,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr"/>
       <c r="C163" t="inlineStr">
         <is>
           <t xml:space="preserve">Сыворотка для лица от морщин с микроиглами 2000 и пдрн/PDRN </t>
@@ -6988,7 +6964,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B164" t="inlineStr"/>
       <c r="C164" t="inlineStr">
         <is>
           <t>Крем для лица увлажняющий капсульный /PDRN PINK COLLAGEN CAP</t>
@@ -7025,7 +7000,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B165" t="inlineStr"/>
       <c r="C165" t="inlineStr">
         <is>
           <t>капсульный крем для лица /TXA NIACINAMIDE CAPSULE CREAM 55g</t>
@@ -7062,7 +7036,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B166" t="inlineStr"/>
       <c r="C166" t="inlineStr">
         <is>
           <t>ROUND LAB STICK POUCH KIT(Набор саше миниатюр для лица 12 шт</t>
@@ -7099,7 +7072,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B167" t="inlineStr"/>
       <c r="C167" t="inlineStr">
         <is>
           <t>CELIMAX ONE STEP BODY BRIGHTENING PAD 60PADS</t>
@@ -7136,7 +7108,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B168" t="inlineStr"/>
       <c r="C168" t="inlineStr">
         <is>
           <t>SKIN1004 Madagascar Centella Tone Brightening Capsule Ampoul</t>
@@ -7173,7 +7144,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B169" t="inlineStr"/>
       <c r="C169" t="inlineStr">
         <is>
           <t>CELIMAX THE REAL NONI ENERGY REPAIR CREAM 50ML</t>
@@ -7210,7 +7180,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B170" t="inlineStr"/>
       <c r="C170" t="inlineStr">
         <is>
           <t>PDRN PINK HYALURONIC MOISTURIZING CREAM 50ml</t>
@@ -7247,7 +7216,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B171" t="inlineStr"/>
       <c r="C171" t="inlineStr">
         <is>
           <t>Антивозрастная сыворотка-стик для лица с волюфилином</t>
@@ -7284,7 +7252,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B172" t="inlineStr"/>
       <c r="C172" t="inlineStr">
         <is>
           <t>Сыворотка с Ниацинамидом для лица от прыщей Niacinamide/[Der</t>
@@ -7321,7 +7288,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B173" t="inlineStr"/>
       <c r="C173" t="inlineStr">
         <is>
           <t>PINE CALMING CICA PAD_50pcs/Тонер пэды диски для лица от пры</t>
@@ -7358,7 +7324,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B174" t="inlineStr"/>
       <c r="C174" t="inlineStr">
         <is>
           <t>Гидрофильное масло CELIMAX DERMA NATURE FRESH BLACKHEAD JOJO</t>
@@ -7395,7 +7360,6 @@
           <t>НОВЫЕ/ПРОЧЕЕ</t>
         </is>
       </c>
-      <c r="B175" t="inlineStr"/>
       <c r="C175" t="inlineStr">
         <is>
           <t>Тонер пэды для лица,60 шт CELIMAX JI WOO GAE HEARTLEAF BHA P</t>
@@ -7438,4 +7402,1749 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Транзит, мес</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Бренд</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Итого сейчас</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Продажи/мес</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Спрос 2маг/мес</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Хватит дней</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>В контейнер, шт</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Вес, т</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CELIMAX</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>551465879</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CELIMAX THE VITA-A RETINOL SHOT TIGHTENING SERUM [30ml]</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4856</v>
+      </c>
+      <c r="E3" t="n">
+        <v>618</v>
+      </c>
+      <c r="F3">
+        <f>E3*$J$3</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>IF(F3=0,"",ROUND(D3/(F3/30),0))</f>
+        <v/>
+      </c>
+      <c r="H3">
+        <f>MAX(0,ROUND(F3*$J$2-D3,0))</f>
+        <v/>
+      </c>
+      <c r="I3" s="1">
+        <f>H3*$J$4/1000</f>
+        <v/>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ENOUGH</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>238358954</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ENOUGH - Collagen 3in1 Sun Cream SPF50 PA+++ [50ml] / о</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>318</v>
+      </c>
+      <c r="E4" t="n">
+        <v>539</v>
+      </c>
+      <c r="F4">
+        <f>E4*$J$3</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>IF(F4=0,"",ROUND(D4/(F4/30),0))</f>
+        <v/>
+      </c>
+      <c r="H4">
+        <f>MAX(0,ROUND(F4*$J$2-D4,0))</f>
+        <v/>
+      </c>
+      <c r="I4" s="1">
+        <f>H4*$J$4/1000</f>
+        <v/>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ENOUGH</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>207796789</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ENOUGH - Gold Snail Moisture Foundation [Tone 13] / Тон</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1036</v>
+      </c>
+      <c r="E5" t="n">
+        <v>306</v>
+      </c>
+      <c r="F5">
+        <f>E5*$J$3</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>IF(F5=0,"",ROUND(D5/(F5/30),0))</f>
+        <v/>
+      </c>
+      <c r="H5">
+        <f>MAX(0,ROUND(F5*$J$2-D5,0))</f>
+        <v/>
+      </c>
+      <c r="I5" s="1">
+        <f>H5*$J$4/1000</f>
+        <v/>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MANYO</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>198156472</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MANYO - Galac Whitening Vita Serum [50ml] / Осветляющая</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1142</v>
+      </c>
+      <c r="E6" t="n">
+        <v>237</v>
+      </c>
+      <c r="F6">
+        <f>E6*$J$3</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>IF(F6=0,"",ROUND(D6/(F6/30),0))</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>MAX(0,ROUND(F6*$J$2-D6,0))</f>
+        <v/>
+      </c>
+      <c r="I6" s="1">
+        <f>H6*$J$4/1000</f>
+        <v/>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>JIGOTT</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>207483179</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>JIGOTT - Snail Reparing Cream [100ml] / Крем для лица у</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1540</v>
+      </c>
+      <c r="E7" t="n">
+        <v>212</v>
+      </c>
+      <c r="F7">
+        <f>E7*$J$3</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>IF(F7=0,"",ROUND(D7/(F7/30),0))</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>MAX(0,ROUND(F7*$J$2-D7,0))</f>
+        <v/>
+      </c>
+      <c r="I7">
+        <f>H7*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PETITFEE</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>151175880</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PETITFEE - Black Pearl &amp; Gold Hydrogel Eye Patch [60ea]</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1185</v>
+      </c>
+      <c r="E8" t="n">
+        <v>185</v>
+      </c>
+      <c r="F8">
+        <f>E8*$J$3</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IF(F8=0,"",ROUND(D8/(F8/30),0))</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>MAX(0,ROUND(F8*$J$2-D8,0))</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>H8*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ENOUGH</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>207796898</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ENOUGH - Gold Snail Moisture Foundation [Tone 21] / Тон</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>684</v>
+      </c>
+      <c r="E9" t="n">
+        <v>175</v>
+      </c>
+      <c r="F9">
+        <f>E9*$J$3</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>IF(F9=0,"",ROUND(D9/(F9/30),0))</f>
+        <v/>
+      </c>
+      <c r="H9">
+        <f>MAX(0,ROUND(F9*$J$2-D9,0))</f>
+        <v/>
+      </c>
+      <c r="I9">
+        <f>H9*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ELIZAVECCA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>207796563</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ELIZAVECCA - Aqua Hyaluronic Acid Water Drop Cream / Ув</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>45</v>
+      </c>
+      <c r="E10" t="n">
+        <v>171</v>
+      </c>
+      <c r="F10">
+        <f>E10*$J$3</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>IF(F10=0,"",ROUND(D10/(F10/30),0))</f>
+        <v/>
+      </c>
+      <c r="H10">
+        <f>MAX(0,ROUND(F10*$J$2-D10,0))</f>
+        <v/>
+      </c>
+      <c r="I10">
+        <f>H10*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ENOUGH</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>170198337</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ENOUGH - Premium 8 Peptide Full Cover Perfect Foundatio</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>632</v>
+      </c>
+      <c r="E11" t="n">
+        <v>160</v>
+      </c>
+      <c r="F11">
+        <f>E11*$J$3</f>
+        <v/>
+      </c>
+      <c r="G11">
+        <f>IF(F11=0,"",ROUND(D11/(F11/30),0))</f>
+        <v/>
+      </c>
+      <c r="H11">
+        <f>MAX(0,ROUND(F11*$J$2-D11,0))</f>
+        <v/>
+      </c>
+      <c r="I11">
+        <f>H11*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PETITFEE</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>226115324</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PETITFEE - Agave Cooling Hydrogel Face Mask [5pcs] / Ох</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1197</v>
+      </c>
+      <c r="E12" t="n">
+        <v>153</v>
+      </c>
+      <c r="F12">
+        <f>E12*$J$3</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>IF(F12=0,"",ROUND(D12/(F12/30),0))</f>
+        <v/>
+      </c>
+      <c r="H12">
+        <f>MAX(0,ROUND(F12*$J$2-D12,0))</f>
+        <v/>
+      </c>
+      <c r="I12">
+        <f>H12*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ENOUGH</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>170198180</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ENOUGH - Premium Rich Gold Double Wear Radiance Foundat</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>627</v>
+      </c>
+      <c r="E13" t="n">
+        <v>139</v>
+      </c>
+      <c r="F13">
+        <f>E13*$J$3</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>IF(F13=0,"",ROUND(D13/(F13/30),0))</f>
+        <v/>
+      </c>
+      <c r="H13">
+        <f>MAX(0,ROUND(F13*$J$2-D13,0))</f>
+        <v/>
+      </c>
+      <c r="I13">
+        <f>H13*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ENOUGH</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>170198835</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ENOUGH - Premium Ultra X10 Cover Up Collagen Foundation</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E14" t="n">
+        <v>135</v>
+      </c>
+      <c r="F14">
+        <f>E14*$J$3</f>
+        <v/>
+      </c>
+      <c r="G14">
+        <f>IF(F14=0,"",ROUND(D14/(F14/30),0))</f>
+        <v/>
+      </c>
+      <c r="H14">
+        <f>MAX(0,ROUND(F14*$J$2-D14,0))</f>
+        <v/>
+      </c>
+      <c r="I14">
+        <f>H14*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ENOUGH</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>170198109</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ENOUGH - Premium Rich Gold Double Wear Radiance Foundat</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>540</v>
+      </c>
+      <c r="E15" t="n">
+        <v>125</v>
+      </c>
+      <c r="F15">
+        <f>E15*$J$3</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>IF(F15=0,"",ROUND(D15/(F15/30),0))</f>
+        <v/>
+      </c>
+      <c r="H15">
+        <f>MAX(0,ROUND(F15*$J$2-D15,0))</f>
+        <v/>
+      </c>
+      <c r="I15">
+        <f>H15*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ELIZAVECCA</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>207796439</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ELIZAVECCA - Natural 90% Olive Cleansing Oil / Очищающе</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="n">
+        <v>122</v>
+      </c>
+      <c r="F16">
+        <f>E16*$J$3</f>
+        <v/>
+      </c>
+      <c r="G16">
+        <f>IF(F16=0,"",ROUND(D16/(F16/30),0))</f>
+        <v/>
+      </c>
+      <c r="H16">
+        <f>MAX(0,ROUND(F16*$J$2-D16,0))</f>
+        <v/>
+      </c>
+      <c r="I16">
+        <f>H16*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MANYO</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>205054338</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MANYO - Bifida Biome Ampoule Toner [400ml] / Ампульный </t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>112</v>
+      </c>
+      <c r="F17">
+        <f>E17*$J$3</f>
+        <v/>
+      </c>
+      <c r="G17">
+        <f>IF(F17=0,"",ROUND(D17/(F17/30),0))</f>
+        <v/>
+      </c>
+      <c r="H17">
+        <f>MAX(0,ROUND(F17*$J$2-D17,0))</f>
+        <v/>
+      </c>
+      <c r="I17">
+        <f>H17*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>MANYO</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>198156698</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MANYO - Pure Cleansing Oil [200ml] / Гидрофильное масло</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>368</v>
+      </c>
+      <c r="E18" t="n">
+        <v>106</v>
+      </c>
+      <c r="F18">
+        <f>E18*$J$3</f>
+        <v/>
+      </c>
+      <c r="G18">
+        <f>IF(F18=0,"",ROUND(D18/(F18/30),0))</f>
+        <v/>
+      </c>
+      <c r="H18">
+        <f>MAX(0,ROUND(F18*$J$2-D18,0))</f>
+        <v/>
+      </c>
+      <c r="I18">
+        <f>H18*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ELIZAVECCA</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>206057411</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ELIZAVECCA - Hell pore clean up aha fruit toner [ 200ml</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>458</v>
+      </c>
+      <c r="E19" t="n">
+        <v>105</v>
+      </c>
+      <c r="F19">
+        <f>E19*$J$3</f>
+        <v/>
+      </c>
+      <c r="G19">
+        <f>IF(F19=0,"",ROUND(D19/(F19/30),0))</f>
+        <v/>
+      </c>
+      <c r="H19">
+        <f>MAX(0,ROUND(F19*$J$2-D19,0))</f>
+        <v/>
+      </c>
+      <c r="I19">
+        <f>H19*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DEOPROCE</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>214305722</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>DEOPROCE SHAMPOO+BALSAM - BLACK GARLIC[2000ml]</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>570</v>
+      </c>
+      <c r="E20" t="n">
+        <v>95</v>
+      </c>
+      <c r="F20">
+        <f>E20*$J$3</f>
+        <v/>
+      </c>
+      <c r="G20">
+        <f>IF(F20=0,"",ROUND(D20/(F20/30),0))</f>
+        <v/>
+      </c>
+      <c r="H20">
+        <f>MAX(0,ROUND(F20*$J$2-D20,0))</f>
+        <v/>
+      </c>
+      <c r="I20">
+        <f>H20*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ELIZAVECCA</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>190159348</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ELIZAVECCA - 24K Gold Snail Cleansing Foam [180ml] / Зо</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>45</v>
+      </c>
+      <c r="E21" t="n">
+        <v>95</v>
+      </c>
+      <c r="F21">
+        <f>E21*$J$3</f>
+        <v/>
+      </c>
+      <c r="G21">
+        <f>IF(F21=0,"",ROUND(D21/(F21/30),0))</f>
+        <v/>
+      </c>
+      <c r="H21">
+        <f>MAX(0,ROUND(F21*$J$2-D21,0))</f>
+        <v/>
+      </c>
+      <c r="I21">
+        <f>H21*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ENOUGH</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>170198876</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ENOUGH - Premium Ultra X10 Cover Up Collagen Foundation</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>278</v>
+      </c>
+      <c r="E22" t="n">
+        <v>90</v>
+      </c>
+      <c r="F22">
+        <f>E22*$J$3</f>
+        <v/>
+      </c>
+      <c r="G22">
+        <f>IF(F22=0,"",ROUND(D22/(F22/30),0))</f>
+        <v/>
+      </c>
+      <c r="H22">
+        <f>MAX(0,ROUND(F22*$J$2-D22,0))</f>
+        <v/>
+      </c>
+      <c r="I22">
+        <f>H22*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PETITFEE</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>226117746</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>PETITFEE - Chamomile Lightening Hydrogel Mask Pack [5pc</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>129</v>
+      </c>
+      <c r="E23" t="n">
+        <v>88</v>
+      </c>
+      <c r="F23">
+        <f>E23*$J$3</f>
+        <v/>
+      </c>
+      <c r="G23">
+        <f>IF(F23=0,"",ROUND(D23/(F23/30),0))</f>
+        <v/>
+      </c>
+      <c r="H23">
+        <f>MAX(0,ROUND(F23*$J$2-D23,0))</f>
+        <v/>
+      </c>
+      <c r="I23">
+        <f>H23*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EKEL</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>208202076</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>EKEL - Ampule Сream Сollagen [70ml] / Крем для лица амп</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>324</v>
+      </c>
+      <c r="E24" t="n">
+        <v>83</v>
+      </c>
+      <c r="F24">
+        <f>E24*$J$3</f>
+        <v/>
+      </c>
+      <c r="G24">
+        <f>IF(F24=0,"",ROUND(D24/(F24/30),0))</f>
+        <v/>
+      </c>
+      <c r="H24">
+        <f>MAX(0,ROUND(F24*$J$2-D24,0))</f>
+        <v/>
+      </c>
+      <c r="I24">
+        <f>H24*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>437254254</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ROUND LAB SOYBEAN PANTHENOL CREAM_80ml - Крем для лица </t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>310</v>
+      </c>
+      <c r="E25" t="n">
+        <v>72</v>
+      </c>
+      <c r="F25">
+        <f>E25*$J$3</f>
+        <v/>
+      </c>
+      <c r="G25">
+        <f>IF(F25=0,"",ROUND(D25/(F25/30),0))</f>
+        <v/>
+      </c>
+      <c r="H25">
+        <f>MAX(0,ROUND(F25*$J$2-D25,0))</f>
+        <v/>
+      </c>
+      <c r="I25">
+        <f>H25*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>HEIMISH</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>207465786</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>HEIMISH - All Clean Balm Mandarin [120ml] / Очищающий г</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>108</v>
+      </c>
+      <c r="E26" t="n">
+        <v>68</v>
+      </c>
+      <c r="F26">
+        <f>E26*$J$3</f>
+        <v/>
+      </c>
+      <c r="G26">
+        <f>IF(F26=0,"",ROUND(D26/(F26/30),0))</f>
+        <v/>
+      </c>
+      <c r="H26">
+        <f>MAX(0,ROUND(F26*$J$2-D26,0))</f>
+        <v/>
+      </c>
+      <c r="I26">
+        <f>H26*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ETUDEHOUSE</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>154160085</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ETUDE - Baking Powder Crunch Pore Scrub [24*7ml] / Очищ</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>309</v>
+      </c>
+      <c r="E27" t="n">
+        <v>65</v>
+      </c>
+      <c r="F27">
+        <f>E27*$J$3</f>
+        <v/>
+      </c>
+      <c r="G27">
+        <f>IF(F27=0,"",ROUND(D27/(F27/30),0))</f>
+        <v/>
+      </c>
+      <c r="H27">
+        <f>MAX(0,ROUND(F27*$J$2-D27,0))</f>
+        <v/>
+      </c>
+      <c r="I27">
+        <f>H27*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PETITFEE</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>179611318</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PETITFEE - Chamomile Lightening Hydrogel Eye Patch [60e</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>357</v>
+      </c>
+      <c r="E28" t="n">
+        <v>50</v>
+      </c>
+      <c r="F28">
+        <f>E28*$J$3</f>
+        <v/>
+      </c>
+      <c r="G28">
+        <f>IF(F28=0,"",ROUND(D28/(F28/30),0))</f>
+        <v/>
+      </c>
+      <c r="H28">
+        <f>MAX(0,ROUND(F28*$J$2-D28,0))</f>
+        <v/>
+      </c>
+      <c r="I28">
+        <f>H28*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ETUDEHOUSE</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>154159632</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ETUDE - Baking Powder BB Deep Cleansing Foam [30ml] / П</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>175</v>
+      </c>
+      <c r="E29" t="n">
+        <v>50</v>
+      </c>
+      <c r="F29">
+        <f>E29*$J$3</f>
+        <v/>
+      </c>
+      <c r="G29">
+        <f>IF(F29=0,"",ROUND(D29/(F29/30),0))</f>
+        <v/>
+      </c>
+      <c r="H29">
+        <f>MAX(0,ROUND(F29*$J$2-D29,0))</f>
+        <v/>
+      </c>
+      <c r="I29">
+        <f>H29*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>207481251</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>COSRX - Advanced Snail 96 Mucin Power Essence [100ml] /</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>38</v>
+      </c>
+      <c r="E30" t="n">
+        <v>46</v>
+      </c>
+      <c r="F30">
+        <f>E30*$J$3</f>
+        <v/>
+      </c>
+      <c r="G30">
+        <f>IF(F30=0,"",ROUND(D30/(F30/30),0))</f>
+        <v/>
+      </c>
+      <c r="H30">
+        <f>MAX(0,ROUND(F30*$J$2-D30,0))</f>
+        <v/>
+      </c>
+      <c r="I30">
+        <f>H30*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>437797551</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ROUND LAB VITA NIACINAMIDE DARK SPOT SERUM 30ml - Сывор</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>62</v>
+      </c>
+      <c r="E31" t="n">
+        <v>40</v>
+      </c>
+      <c r="F31">
+        <f>E31*$J$3</f>
+        <v/>
+      </c>
+      <c r="G31">
+        <f>IF(F31=0,"",ROUND(D31/(F31/30),0))</f>
+        <v/>
+      </c>
+      <c r="H31">
+        <f>MAX(0,ROUND(F31*$J$2-D31,0))</f>
+        <v/>
+      </c>
+      <c r="I31">
+        <f>H31*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>DEOPROCE</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>608837066</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>DEOPROCE SHAMPOO - BLACK GARLIC INTENSME ENERGY [600ml]</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>122</v>
+      </c>
+      <c r="E32" t="n">
+        <v>39</v>
+      </c>
+      <c r="F32">
+        <f>E32*$J$3</f>
+        <v/>
+      </c>
+      <c r="G32">
+        <f>IF(F32=0,"",ROUND(D32/(F32/30),0))</f>
+        <v/>
+      </c>
+      <c r="H32">
+        <f>MAX(0,ROUND(F32*$J$2-D32,0))</f>
+        <v/>
+      </c>
+      <c r="I32">
+        <f>H32*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ENOUGH</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>611747838</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ENOUGH - Collagen Moisture Foundation [Tone 23] / Тонал</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>90</v>
+      </c>
+      <c r="E33" t="n">
+        <v>34</v>
+      </c>
+      <c r="F33">
+        <f>E33*$J$3</f>
+        <v/>
+      </c>
+      <c r="G33">
+        <f>IF(F33=0,"",ROUND(D33/(F33/30),0))</f>
+        <v/>
+      </c>
+      <c r="H33">
+        <f>MAX(0,ROUND(F33*$J$2-D33,0))</f>
+        <v/>
+      </c>
+      <c r="I33">
+        <f>H33*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>JIGOTT</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>212753217</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>JIGOTT - Collagen Healing Cream [100ml] / Крем для лица</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>133</v>
+      </c>
+      <c r="E34" t="n">
+        <v>31</v>
+      </c>
+      <c r="F34">
+        <f>E34*$J$3</f>
+        <v/>
+      </c>
+      <c r="G34">
+        <f>IF(F34=0,"",ROUND(D34/(F34/30),0))</f>
+        <v/>
+      </c>
+      <c r="H34">
+        <f>MAX(0,ROUND(F34*$J$2-D34,0))</f>
+        <v/>
+      </c>
+      <c r="I34">
+        <f>H34*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>437776835</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ROUND LAB PINE CALMING CICA AMPOULE_30ml - Сыворотка дл</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>103</v>
+      </c>
+      <c r="E35" t="n">
+        <v>31</v>
+      </c>
+      <c r="F35">
+        <f>E35*$J$3</f>
+        <v/>
+      </c>
+      <c r="G35">
+        <f>IF(F35=0,"",ROUND(D35/(F35/30),0))</f>
+        <v/>
+      </c>
+      <c r="H35">
+        <f>MAX(0,ROUND(F35*$J$2-D35,0))</f>
+        <v/>
+      </c>
+      <c r="I35">
+        <f>H35*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DEOPROCE</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>608624295</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>DEOPROCE SHAMPOO - BLACK GARLIC INTENSME ENERGY [600ml]</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>143</v>
+      </c>
+      <c r="E36" t="n">
+        <v>30</v>
+      </c>
+      <c r="F36">
+        <f>E36*$J$3</f>
+        <v/>
+      </c>
+      <c r="G36">
+        <f>IF(F36=0,"",ROUND(D36/(F36/30),0))</f>
+        <v/>
+      </c>
+      <c r="H36">
+        <f>MAX(0,ROUND(F36*$J$2-D36,0))</f>
+        <v/>
+      </c>
+      <c r="I36">
+        <f>H36*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>DEOPROCE</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>214304883</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>DEOPROCE - SNAIL RECOVERY CREAM [100g] / Крем восстанав</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>57</v>
+      </c>
+      <c r="E37" t="n">
+        <v>22</v>
+      </c>
+      <c r="F37">
+        <f>E37*$J$3</f>
+        <v/>
+      </c>
+      <c r="G37">
+        <f>IF(F37=0,"",ROUND(D37/(F37/30),0))</f>
+        <v/>
+      </c>
+      <c r="H37">
+        <f>MAX(0,ROUND(F37*$J$2-D37,0))</f>
+        <v/>
+      </c>
+      <c r="I37">
+        <f>H37*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>TheOrdinary</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>214312385</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>THE ORDINARY - Argireline Solution 10% [30ml] / Сыворот</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>127</v>
+      </c>
+      <c r="E38" t="n">
+        <v>22</v>
+      </c>
+      <c r="F38">
+        <f>E38*$J$3</f>
+        <v/>
+      </c>
+      <c r="G38">
+        <f>IF(F38=0,"",ROUND(D38/(F38/30),0))</f>
+        <v/>
+      </c>
+      <c r="H38">
+        <f>MAX(0,ROUND(F38*$J$2-D38,0))</f>
+        <v/>
+      </c>
+      <c r="I38">
+        <f>H38*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PETITFEE</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>180992464</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>PETITFEE - Aura Quartz Hydrogel Eye Patch [60ea]</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>126</v>
+      </c>
+      <c r="E39" t="n">
+        <v>20</v>
+      </c>
+      <c r="F39">
+        <f>E39*$J$3</f>
+        <v/>
+      </c>
+      <c r="G39">
+        <f>IF(F39=0,"",ROUND(D39/(F39/30),0))</f>
+        <v/>
+      </c>
+      <c r="H39">
+        <f>MAX(0,ROUND(F39*$J$2-D39,0))</f>
+        <v/>
+      </c>
+      <c r="I39">
+        <f>H39*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LEBELAGE</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>207818642</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>LEBELAGE - Dr. Hyaluronic Derma Eye Cream [40ml] / Крем</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>39</v>
+      </c>
+      <c r="E40" t="n">
+        <v>19</v>
+      </c>
+      <c r="F40">
+        <f>E40*$J$3</f>
+        <v/>
+      </c>
+      <c r="G40">
+        <f>IF(F40=0,"",ROUND(D40/(F40/30),0))</f>
+        <v/>
+      </c>
+      <c r="H40">
+        <f>MAX(0,ROUND(F40*$J$2-D40,0))</f>
+        <v/>
+      </c>
+      <c r="I40">
+        <f>H40*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ISNTREE</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>207818000</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ISNTREE - Chestnut AHA 8% Clear Essence Sample [20ml] /</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>60</v>
+      </c>
+      <c r="E41" t="n">
+        <v>15</v>
+      </c>
+      <c r="F41">
+        <f>E41*$J$3</f>
+        <v/>
+      </c>
+      <c r="G41">
+        <f>IF(F41=0,"",ROUND(D41/(F41/30),0))</f>
+        <v/>
+      </c>
+      <c r="H41">
+        <f>MAX(0,ROUND(F41*$J$2-D41,0))</f>
+        <v/>
+      </c>
+      <c r="I41">
+        <f>H41*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>437850261</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ROUND LAB SOYBEAN CLEANSING OIL_200ml - Гидрофильное ма</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>30</v>
+      </c>
+      <c r="E42" t="n">
+        <v>14</v>
+      </c>
+      <c r="F42">
+        <f>E42*$J$3</f>
+        <v/>
+      </c>
+      <c r="G42">
+        <f>IF(F42=0,"",ROUND(D42/(F42/30),0))</f>
+        <v/>
+      </c>
+      <c r="H42">
+        <f>MAX(0,ROUND(F42*$J$2-D42,0))</f>
+        <v/>
+      </c>
+      <c r="I42">
+        <f>H42*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ENOUGH</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>611744611</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ENOUGH Collagen whitening cover tip concealer #02 [9g]/</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E43" t="n">
+        <v>8</v>
+      </c>
+      <c r="F43">
+        <f>E43*$J$3</f>
+        <v/>
+      </c>
+      <c r="G43">
+        <f>IF(F43=0,"",ROUND(D43/(F43/30),0))</f>
+        <v/>
+      </c>
+      <c r="H43">
+        <f>MAX(0,ROUND(F43*$J$2-D43,0))</f>
+        <v/>
+      </c>
+      <c r="I43">
+        <f>H43*$J$4/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="H44" s="1">
+        <f>SUM(H3:H43)</f>
+        <v/>
+      </c>
+      <c r="I44" s="1">
+        <f>SUM(I3:I43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Проверка веса, т</t>
+        </is>
+      </c>
+      <c r="D46">
+        <f>I44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Проверка штук</t>
+        </is>
+      </c>
+      <c r="D47">
+        <f>H44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>FarmStay исключён. Контейнер = позиции с покрытием &lt;150 дней, докуп до 6 мес спроса 2 магазинов.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="G3:G43">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>90</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
coverage: container sheet in заказ 22.06 format with formulas
Container tab rebuilt with the same 12 columns as the заказ 22.06 sheet
(Бренд, Название, Баркод, кол-во, цена, сумма, в коробе, Объем короба, Вес
короба кг, Коробок в заказ, Объем, Вес кг). Formulas: сумма=кол-во×цена,
коробок=ROUNDUP(кол-во/в коробе), объём/вес from box counts. Price/box
pulled from заказ 22.06 by barcode where present; others yellow for input.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XzNBEf4vaaEHRqeR8ZkfFA
</commit_message>
<xml_diff>
--- a/outputs/coverage/pokrytie_po_brendam_2026-06-30.xlsx
+++ b/outputs/coverage/pokrytie_po_brendam_2026-06-30.xlsx
@@ -78,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -89,6 +89,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7410,120 +7413,163 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Транзит, мес</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="n">
-        <v>2</v>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Бренд</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Баркод</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>кол-во</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>цена</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>сумма</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>в коробе</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Объем короба</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Вес короба кг</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>Коробок в заказ</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>Объем</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>Вес кг</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Бренд</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Артикул</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Название</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Итого сейчас</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Продажи/мес</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Спрос 2маг/мес</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>Хватит дней</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>В контейнер, шт</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>Вес, т</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>6</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CELIMAX</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CELIMAX THE VITA-A RETINOL SHOT TIGHTENING SERUM [30ml]/Сыво</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>8809700320805</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1266</v>
+      </c>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2">
+        <f>D2*E2</f>
+        <v/>
+      </c>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2">
+        <f>IF(G2="","",ROUNDUP(D2/G2,0))</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>IF(J2="","",J2*H2)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>IF(J2="","",J2*I2)</f>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CELIMAX</t>
+          <t>ENOUGH</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>551465879</t>
+          <t>ENOUGH - Collagen 3in1 Sun Cream SPF50 PA+++ [50ml] / отбели</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CELIMAX THE VITA-A RETINOL SHOT TIGHTENING SERUM [30ml]</t>
+          <t>8809755462130</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4856</v>
-      </c>
-      <c r="E3" t="n">
-        <v>618</v>
-      </c>
+        <v>5018</v>
+      </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3">
-        <f>E3*$J$3</f>
-        <v/>
-      </c>
-      <c r="G3">
-        <f>IF(F3=0,"",ROUND(D3/(F3/30),0))</f>
-        <v/>
-      </c>
-      <c r="H3">
-        <f>MAX(0,ROUND(F3*$J$2-D3,0))</f>
-        <v/>
-      </c>
-      <c r="I3" s="1">
-        <f>H3*$J$4/1000</f>
-        <v/>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>1.65</v>
+        <f>D3*E3</f>
+        <v/>
+      </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3">
+        <f>IF(G3="","",ROUNDUP(D3/G3,0))</f>
+        <v/>
+      </c>
+      <c r="K3">
+        <f>IF(J3="","",J3*H3)</f>
+        <v/>
+      </c>
+      <c r="L3">
+        <f>IF(J3="","",J3*I3)</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -7534,355 +7580,355 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>238358954</t>
+          <t>ENOUGH - Gold Snail Moisture Foundation [Tone 13] / Тональны</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ENOUGH - Collagen 3in1 Sun Cream SPF50 PA+++ [50ml] / о</t>
+          <t>8809474498809</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>318</v>
-      </c>
-      <c r="E4" t="n">
-        <v>539</v>
-      </c>
+        <v>1990</v>
+      </c>
+      <c r="E4" s="2" t="n"/>
       <c r="F4">
-        <f>E4*$J$3</f>
-        <v/>
-      </c>
-      <c r="G4">
-        <f>IF(F4=0,"",ROUND(D4/(F4/30),0))</f>
-        <v/>
-      </c>
-      <c r="H4">
-        <f>MAX(0,ROUND(F4*$J$2-D4,0))</f>
-        <v/>
-      </c>
-      <c r="I4" s="1">
-        <f>H4*$J$4/1000</f>
-        <v/>
-      </c>
-      <c r="J4" s="2" t="n">
-        <v>0.35</v>
+        <f>D4*E4</f>
+        <v/>
+      </c>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4">
+        <f>IF(G4="","",ROUNDUP(D4/G4,0))</f>
+        <v/>
+      </c>
+      <c r="K4">
+        <f>IF(J4="","",J4*H4)</f>
+        <v/>
+      </c>
+      <c r="L4">
+        <f>IF(J4="","",J4*I4)</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ENOUGH</t>
+          <t>MANYO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>207796789</t>
+          <t>MANYO - Galac Whitening Vita Serum [50ml] / Осветляющая сыво</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ENOUGH - Gold Snail Moisture Foundation [Tone 13] / Тон</t>
+          <t>8809730952014</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1036</v>
-      </c>
-      <c r="E5" t="n">
-        <v>306</v>
-      </c>
+        <v>1204</v>
+      </c>
+      <c r="E5" s="2" t="n"/>
       <c r="F5">
-        <f>E5*$J$3</f>
-        <v/>
-      </c>
-      <c r="G5">
-        <f>IF(F5=0,"",ROUND(D5/(F5/30),0))</f>
-        <v/>
-      </c>
-      <c r="H5">
-        <f>MAX(0,ROUND(F5*$J$2-D5,0))</f>
-        <v/>
-      </c>
-      <c r="I5" s="1">
-        <f>H5*$J$4/1000</f>
-        <v/>
-      </c>
-      <c r="J5" s="2" t="n">
-        <v>26</v>
+        <f>D5*E5</f>
+        <v/>
+      </c>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5">
+        <f>IF(G5="","",ROUNDUP(D5/G5,0))</f>
+        <v/>
+      </c>
+      <c r="K5">
+        <f>IF(J5="","",J5*H5)</f>
+        <v/>
+      </c>
+      <c r="L5">
+        <f>IF(J5="","",J5*I5)</f>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MANYO</t>
+          <t>JIGOTT</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>198156472</t>
+          <t>JIGOTT - Snail Reparing Cream [100ml] / Крем для лица увлажн</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MANYO - Galac Whitening Vita Serum [50ml] / Осветляющая</t>
+          <t>8809210036517</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1142</v>
-      </c>
-      <c r="E6" t="n">
-        <v>237</v>
-      </c>
+        <v>562</v>
+      </c>
+      <c r="E6" s="2" t="n"/>
       <c r="F6">
-        <f>E6*$J$3</f>
-        <v/>
-      </c>
-      <c r="G6">
-        <f>IF(F6=0,"",ROUND(D6/(F6/30),0))</f>
-        <v/>
-      </c>
-      <c r="H6">
-        <f>MAX(0,ROUND(F6*$J$2-D6,0))</f>
-        <v/>
-      </c>
-      <c r="I6" s="1">
-        <f>H6*$J$4/1000</f>
-        <v/>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>120000</v>
+        <f>D6*E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6">
+        <f>IF(G6="","",ROUNDUP(D6/G6,0))</f>
+        <v/>
+      </c>
+      <c r="K6">
+        <f>IF(J6="","",J6*H6)</f>
+        <v/>
+      </c>
+      <c r="L6">
+        <f>IF(J6="","",J6*I6)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JIGOTT</t>
+          <t>PETITFEE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>207483179</t>
+          <t>PETITFEE - Black Pearl &amp; Gold Hydrogel Eye Patch [60ea] / Ги</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>JIGOTT - Snail Reparing Cream [100ml] / Крем для лица у</t>
+          <t>8809239801820</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1540</v>
-      </c>
-      <c r="E7" t="n">
-        <v>212</v>
-      </c>
+        <v>643</v>
+      </c>
+      <c r="E7" s="2" t="n"/>
       <c r="F7">
-        <f>E7*$J$3</f>
-        <v/>
-      </c>
-      <c r="G7">
-        <f>IF(F7=0,"",ROUND(D7/(F7/30),0))</f>
-        <v/>
-      </c>
-      <c r="H7">
-        <f>MAX(0,ROUND(F7*$J$2-D7,0))</f>
-        <v/>
-      </c>
-      <c r="I7">
-        <f>H7*$J$4/1000</f>
+        <f>D7*E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7">
+        <f>IF(G7="","",ROUNDUP(D7/G7,0))</f>
+        <v/>
+      </c>
+      <c r="K7">
+        <f>IF(J7="","",J7*H7)</f>
+        <v/>
+      </c>
+      <c r="L7">
+        <f>IF(J7="","",J7*I7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PETITFEE</t>
+          <t>ENOUGH</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>151175880</t>
+          <t>ENOUGH - Gold Snail Moisture Foundation [Tone 21] / Тональны</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PETITFEE - Black Pearl &amp; Gold Hydrogel Eye Patch [60ea]</t>
+          <t>8809474498816</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1185</v>
-      </c>
-      <c r="E8" t="n">
-        <v>185</v>
-      </c>
+        <v>1048</v>
+      </c>
+      <c r="E8" s="2" t="n"/>
       <c r="F8">
-        <f>E8*$J$3</f>
-        <v/>
-      </c>
-      <c r="G8">
-        <f>IF(F8=0,"",ROUND(D8/(F8/30),0))</f>
-        <v/>
-      </c>
-      <c r="H8">
-        <f>MAX(0,ROUND(F8*$J$2-D8,0))</f>
-        <v/>
-      </c>
-      <c r="I8">
-        <f>H8*$J$4/1000</f>
+        <f>D8*E8</f>
+        <v/>
+      </c>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8">
+        <f>IF(G8="","",ROUNDUP(D8/G8,0))</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IF(J8="","",J8*H8)</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IF(J8="","",J8*I8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ENOUGH</t>
+          <t>ELIZAVECCA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>207796898</t>
+          <t>ELIZAVECCA - Aqua Hyaluronic Acid Water Drop Cream / Увлажня</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ENOUGH - Gold Snail Moisture Foundation [Tone 21] / Тон</t>
+          <t>8809418750505</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>684</v>
-      </c>
-      <c r="E9" t="n">
-        <v>175</v>
-      </c>
+        <v>1651</v>
+      </c>
+      <c r="E9" s="2" t="n"/>
       <c r="F9">
-        <f>E9*$J$3</f>
-        <v/>
-      </c>
-      <c r="G9">
-        <f>IF(F9=0,"",ROUND(D9/(F9/30),0))</f>
-        <v/>
-      </c>
-      <c r="H9">
-        <f>MAX(0,ROUND(F9*$J$2-D9,0))</f>
-        <v/>
-      </c>
-      <c r="I9">
-        <f>H9*$J$4/1000</f>
+        <f>D9*E9</f>
+        <v/>
+      </c>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9">
+        <f>IF(G9="","",ROUNDUP(D9/G9,0))</f>
+        <v/>
+      </c>
+      <c r="K9">
+        <f>IF(J9="","",J9*H9)</f>
+        <v/>
+      </c>
+      <c r="L9">
+        <f>IF(J9="","",J9*I9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ELIZAVECCA</t>
+          <t>ENOUGH</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>207796563</t>
+          <t>ENOUGH - Premium 8 Peptide Full Cover Perfect Foundation [To</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ELIZAVECCA - Aqua Hyaluronic Acid Water Drop Cream / Ув</t>
+          <t>8809605870979</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>45</v>
-      </c>
-      <c r="E10" t="n">
-        <v>171</v>
-      </c>
+        <v>955</v>
+      </c>
+      <c r="E10" s="2" t="n"/>
       <c r="F10">
-        <f>E10*$J$3</f>
-        <v/>
-      </c>
-      <c r="G10">
-        <f>IF(F10=0,"",ROUND(D10/(F10/30),0))</f>
-        <v/>
-      </c>
-      <c r="H10">
-        <f>MAX(0,ROUND(F10*$J$2-D10,0))</f>
-        <v/>
-      </c>
-      <c r="I10">
-        <f>H10*$J$4/1000</f>
+        <f>D10*E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10">
+        <f>IF(G10="","",ROUNDUP(D10/G10,0))</f>
+        <v/>
+      </c>
+      <c r="K10">
+        <f>IF(J10="","",J10*H10)</f>
+        <v/>
+      </c>
+      <c r="L10">
+        <f>IF(J10="","",J10*I10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ENOUGH</t>
+          <t>PETITFEE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>170198337</t>
+          <t>PETITFEE - Agave Cooling Hydrogel Face Mask [5pcs] / Охлажда</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ENOUGH - Premium 8 Peptide Full Cover Perfect Foundatio</t>
+          <t>8809508850443</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>632</v>
-      </c>
-      <c r="E11" t="n">
-        <v>160</v>
-      </c>
+        <v>321</v>
+      </c>
+      <c r="E11" s="2" t="n"/>
       <c r="F11">
-        <f>E11*$J$3</f>
-        <v/>
-      </c>
-      <c r="G11">
-        <f>IF(F11=0,"",ROUND(D11/(F11/30),0))</f>
-        <v/>
-      </c>
-      <c r="H11">
-        <f>MAX(0,ROUND(F11*$J$2-D11,0))</f>
-        <v/>
-      </c>
-      <c r="I11">
-        <f>H11*$J$4/1000</f>
+        <f>D11*E11</f>
+        <v/>
+      </c>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11">
+        <f>IF(G11="","",ROUNDUP(D11/G11,0))</f>
+        <v/>
+      </c>
+      <c r="K11">
+        <f>IF(J11="","",J11*H11)</f>
+        <v/>
+      </c>
+      <c r="L11">
+        <f>IF(J11="","",J11*I11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PETITFEE</t>
+          <t>ENOUGH</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>226115324</t>
+          <t>ENOUGH - Premium Rich Gold Double Wear Radiance Foundation [</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PETITFEE - Agave Cooling Hydrogel Face Mask [5pcs] / Ох</t>
+          <t>8809605871938</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1197</v>
-      </c>
-      <c r="E12" t="n">
-        <v>153</v>
-      </c>
+        <v>749</v>
+      </c>
+      <c r="E12" s="2" t="n"/>
       <c r="F12">
-        <f>E12*$J$3</f>
-        <v/>
-      </c>
-      <c r="G12">
-        <f>IF(F12=0,"",ROUND(D12/(F12/30),0))</f>
-        <v/>
-      </c>
-      <c r="H12">
-        <f>MAX(0,ROUND(F12*$J$2-D12,0))</f>
-        <v/>
-      </c>
-      <c r="I12">
-        <f>H12*$J$4/1000</f>
+        <f>D12*E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12">
+        <f>IF(G12="","",ROUNDUP(D12/G12,0))</f>
+        <v/>
+      </c>
+      <c r="K12">
+        <f>IF(J12="","",J12*H12)</f>
+        <v/>
+      </c>
+      <c r="L12">
+        <f>IF(J12="","",J12*I12)</f>
         <v/>
       </c>
     </row>
@@ -7894,34 +7940,35 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>170198180</t>
+          <t>ENOUGH - Premium Ultra X10 Cover Up Collagen Foundation [Ton</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ENOUGH - Premium Rich Gold Double Wear Radiance Foundat</t>
+          <t>8809605870993</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>627</v>
-      </c>
-      <c r="E13" t="n">
-        <v>139</v>
-      </c>
+        <v>333</v>
+      </c>
+      <c r="E13" s="2" t="n"/>
       <c r="F13">
-        <f>E13*$J$3</f>
-        <v/>
-      </c>
-      <c r="G13">
-        <f>IF(F13=0,"",ROUND(D13/(F13/30),0))</f>
-        <v/>
-      </c>
-      <c r="H13">
-        <f>MAX(0,ROUND(F13*$J$2-D13,0))</f>
-        <v/>
-      </c>
-      <c r="I13">
-        <f>H13*$J$4/1000</f>
+        <f>D13*E13</f>
+        <v/>
+      </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13">
+        <f>IF(G13="","",ROUNDUP(D13/G13,0))</f>
+        <v/>
+      </c>
+      <c r="K13">
+        <f>IF(J13="","",J13*H13)</f>
+        <v/>
+      </c>
+      <c r="L13">
+        <f>IF(J13="","",J13*I13)</f>
         <v/>
       </c>
     </row>
@@ -7933,112 +7980,115 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>170198835</t>
+          <t>ENOUGH - Premium Rich Gold Double Wear Radiance Foundation [</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ENOUGH - Premium Ultra X10 Cover Up Collagen Foundation</t>
+          <t>8809605871945</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E14" t="n">
-        <v>135</v>
-      </c>
+        <v>698</v>
+      </c>
+      <c r="E14" s="2" t="n"/>
       <c r="F14">
-        <f>E14*$J$3</f>
-        <v/>
-      </c>
-      <c r="G14">
-        <f>IF(F14=0,"",ROUND(D14/(F14/30),0))</f>
-        <v/>
-      </c>
-      <c r="H14">
-        <f>MAX(0,ROUND(F14*$J$2-D14,0))</f>
-        <v/>
-      </c>
-      <c r="I14">
-        <f>H14*$J$4/1000</f>
+        <f>D14*E14</f>
+        <v/>
+      </c>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14">
+        <f>IF(G14="","",ROUNDUP(D14/G14,0))</f>
+        <v/>
+      </c>
+      <c r="K14">
+        <f>IF(J14="","",J14*H14)</f>
+        <v/>
+      </c>
+      <c r="L14">
+        <f>IF(J14="","",J14*I14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ENOUGH</t>
+          <t>ELIZAVECCA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>170198109</t>
+          <t>ELIZAVECCA - Natural 90% Olive Cleansing Oil / Очищающее гид</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ENOUGH - Premium Rich Gold Double Wear Radiance Foundat</t>
+          <t>8809071365504</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>540</v>
-      </c>
-      <c r="E15" t="n">
-        <v>125</v>
-      </c>
+        <v>1203</v>
+      </c>
+      <c r="E15" s="2" t="n"/>
       <c r="F15">
-        <f>E15*$J$3</f>
-        <v/>
-      </c>
-      <c r="G15">
-        <f>IF(F15=0,"",ROUND(D15/(F15/30),0))</f>
-        <v/>
-      </c>
-      <c r="H15">
-        <f>MAX(0,ROUND(F15*$J$2-D15,0))</f>
-        <v/>
-      </c>
-      <c r="I15">
-        <f>H15*$J$4/1000</f>
+        <f>D15*E15</f>
+        <v/>
+      </c>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15">
+        <f>IF(G15="","",ROUNDUP(D15/G15,0))</f>
+        <v/>
+      </c>
+      <c r="K15">
+        <f>IF(J15="","",J15*H15)</f>
+        <v/>
+      </c>
+      <c r="L15">
+        <f>IF(J15="","",J15*I15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ELIZAVECCA</t>
+          <t>MANYO</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>207796439</t>
+          <t>MANYO - Bifida Biome Ampoule Toner [400ml] / Ампульный укреп</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ELIZAVECCA - Natural 90% Olive Cleansing Oil / Очищающе</t>
+          <t>8809657114137</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
-      </c>
-      <c r="E16" t="n">
-        <v>122</v>
-      </c>
+        <v>1111</v>
+      </c>
+      <c r="E16" s="2" t="n"/>
       <c r="F16">
-        <f>E16*$J$3</f>
-        <v/>
-      </c>
-      <c r="G16">
-        <f>IF(F16=0,"",ROUND(D16/(F16/30),0))</f>
-        <v/>
-      </c>
-      <c r="H16">
-        <f>MAX(0,ROUND(F16*$J$2-D16,0))</f>
-        <v/>
-      </c>
-      <c r="I16">
-        <f>H16*$J$4/1000</f>
+        <f>D16*E16</f>
+        <v/>
+      </c>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16">
+        <f>IF(G16="","",ROUNDUP(D16/G16,0))</f>
+        <v/>
+      </c>
+      <c r="K16">
+        <f>IF(J16="","",J16*H16)</f>
+        <v/>
+      </c>
+      <c r="L16">
+        <f>IF(J16="","",J16*I16)</f>
         <v/>
       </c>
     </row>
@@ -8050,736 +8100,759 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>205054338</t>
+          <t xml:space="preserve">MANYO - Pure Cleansing Oil [200ml] / Гидрофильное масло для </t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANYO - Bifida Biome Ampoule Toner [400ml] / Ампульный </t>
+          <t>8809082392292</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="n">
-        <v>112</v>
-      </c>
+        <v>678</v>
+      </c>
+      <c r="E17" s="2" t="n"/>
       <c r="F17">
-        <f>E17*$J$3</f>
-        <v/>
-      </c>
-      <c r="G17">
-        <f>IF(F17=0,"",ROUND(D17/(F17/30),0))</f>
-        <v/>
-      </c>
-      <c r="H17">
-        <f>MAX(0,ROUND(F17*$J$2-D17,0))</f>
-        <v/>
-      </c>
-      <c r="I17">
-        <f>H17*$J$4/1000</f>
+        <f>D17*E17</f>
+        <v/>
+      </c>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17">
+        <f>IF(G17="","",ROUNDUP(D17/G17,0))</f>
+        <v/>
+      </c>
+      <c r="K17">
+        <f>IF(J17="","",J17*H17)</f>
+        <v/>
+      </c>
+      <c r="L17">
+        <f>IF(J17="","",J17*I17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MANYO</t>
+          <t>ELIZAVECCA</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>198156698</t>
+          <t>ELIZAVECCA - Hell pore clean up aha fruit toner [ 200ml] / П</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MANYO - Pure Cleansing Oil [200ml] / Гидрофильное масло</t>
+          <t>8809339907910</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>368</v>
-      </c>
-      <c r="E18" t="n">
-        <v>106</v>
-      </c>
+        <v>578</v>
+      </c>
+      <c r="E18" s="2" t="n"/>
       <c r="F18">
-        <f>E18*$J$3</f>
-        <v/>
-      </c>
-      <c r="G18">
-        <f>IF(F18=0,"",ROUND(D18/(F18/30),0))</f>
-        <v/>
-      </c>
-      <c r="H18">
-        <f>MAX(0,ROUND(F18*$J$2-D18,0))</f>
-        <v/>
-      </c>
-      <c r="I18">
-        <f>H18*$J$4/1000</f>
+        <f>D18*E18</f>
+        <v/>
+      </c>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18">
+        <f>IF(G18="","",ROUNDUP(D18/G18,0))</f>
+        <v/>
+      </c>
+      <c r="K18">
+        <f>IF(J18="","",J18*H18)</f>
+        <v/>
+      </c>
+      <c r="L18">
+        <f>IF(J18="","",J18*I18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ELIZAVECCA</t>
+          <t>DEOPROCE</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>206057411</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>ELIZAVECCA - Hell pore clean up aha fruit toner [ 200ml</t>
-        </is>
-      </c>
+          <t>DEOPROCE SHAMPOO+BALSAM - BLACK GARLIC[2000ml]</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>458</v>
-      </c>
-      <c r="E19" t="n">
-        <v>105</v>
-      </c>
+        <v>374</v>
+      </c>
+      <c r="E19" s="2" t="n"/>
       <c r="F19">
-        <f>E19*$J$3</f>
-        <v/>
-      </c>
-      <c r="G19">
-        <f>IF(F19=0,"",ROUND(D19/(F19/30),0))</f>
-        <v/>
-      </c>
-      <c r="H19">
-        <f>MAX(0,ROUND(F19*$J$2-D19,0))</f>
-        <v/>
-      </c>
-      <c r="I19">
-        <f>H19*$J$4/1000</f>
+        <f>D19*E19</f>
+        <v/>
+      </c>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19">
+        <f>IF(G19="","",ROUNDUP(D19/G19,0))</f>
+        <v/>
+      </c>
+      <c r="K19">
+        <f>IF(J19="","",J19*H19)</f>
+        <v/>
+      </c>
+      <c r="L19">
+        <f>IF(J19="","",J19*I19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>DEOPROCE</t>
+          <t>ELIZAVECCA</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>214305722</t>
+          <t>ELIZAVECCA - 24K Gold Snail Cleansing Foam [180ml] / Золотая</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DEOPROCE SHAMPOO+BALSAM - BLACK GARLIC[2000ml]</t>
+          <t>8809418750338</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>570</v>
-      </c>
-      <c r="E20" t="n">
-        <v>95</v>
-      </c>
+        <v>896</v>
+      </c>
+      <c r="E20" s="2" t="n"/>
       <c r="F20">
-        <f>E20*$J$3</f>
-        <v/>
-      </c>
-      <c r="G20">
-        <f>IF(F20=0,"",ROUND(D20/(F20/30),0))</f>
-        <v/>
-      </c>
-      <c r="H20">
-        <f>MAX(0,ROUND(F20*$J$2-D20,0))</f>
-        <v/>
-      </c>
-      <c r="I20">
-        <f>H20*$J$4/1000</f>
+        <f>D20*E20</f>
+        <v/>
+      </c>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20">
+        <f>IF(G20="","",ROUNDUP(D20/G20,0))</f>
+        <v/>
+      </c>
+      <c r="K20">
+        <f>IF(J20="","",J20*H20)</f>
+        <v/>
+      </c>
+      <c r="L20">
+        <f>IF(J20="","",J20*I20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ELIZAVECCA</t>
+          <t>ENOUGH</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>190159348</t>
+          <t>ENOUGH - Premium Ultra X10 Cover Up Collagen Foundation [Ton</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ELIZAVECCA - 24K Gold Snail Cleansing Foam [180ml] / Зо</t>
+          <t>8809605871006</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>45</v>
+        <v>610</v>
       </c>
       <c r="E21" t="n">
-        <v>95</v>
+        <v>3880</v>
       </c>
       <c r="F21">
-        <f>E21*$J$3</f>
-        <v/>
-      </c>
-      <c r="G21">
-        <f>IF(F21=0,"",ROUND(D21/(F21/30),0))</f>
-        <v/>
-      </c>
-      <c r="H21">
-        <f>MAX(0,ROUND(F21*$J$2-D21,0))</f>
-        <v/>
-      </c>
-      <c r="I21">
-        <f>H21*$J$4/1000</f>
+        <f>D21*E21</f>
+        <v/>
+      </c>
+      <c r="G21" t="n">
+        <v>100</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.0314</v>
+      </c>
+      <c r="I21" t="n">
+        <v>15</v>
+      </c>
+      <c r="J21">
+        <f>IF(G21="","",ROUNDUP(D21/G21,0))</f>
+        <v/>
+      </c>
+      <c r="K21">
+        <f>IF(J21="","",J21*H21)</f>
+        <v/>
+      </c>
+      <c r="L21">
+        <f>IF(J21="","",J21*I21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ENOUGH</t>
+          <t>PETITFEE</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>170198876</t>
+          <t xml:space="preserve">PETITFEE - Chamomile Lightening Hydrogel Mask Pack [5pcs] / </t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ENOUGH - Premium Ultra X10 Cover Up Collagen Foundation</t>
+          <t>8809508850436</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>278</v>
-      </c>
-      <c r="E22" t="n">
-        <v>90</v>
-      </c>
+        <v>745</v>
+      </c>
+      <c r="E22" s="2" t="n"/>
       <c r="F22">
-        <f>E22*$J$3</f>
-        <v/>
-      </c>
-      <c r="G22">
-        <f>IF(F22=0,"",ROUND(D22/(F22/30),0))</f>
-        <v/>
-      </c>
-      <c r="H22">
-        <f>MAX(0,ROUND(F22*$J$2-D22,0))</f>
-        <v/>
-      </c>
-      <c r="I22">
-        <f>H22*$J$4/1000</f>
+        <f>D22*E22</f>
+        <v/>
+      </c>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22">
+        <f>IF(G22="","",ROUNDUP(D22/G22,0))</f>
+        <v/>
+      </c>
+      <c r="K22">
+        <f>IF(J22="","",J22*H22)</f>
+        <v/>
+      </c>
+      <c r="L22">
+        <f>IF(J22="","",J22*I22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PETITFEE</t>
+          <t>EKEL</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>226117746</t>
+          <t>EKEL - Ampule Сream Сollagen [70ml] / Крем для лица ампульны</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PETITFEE - Chamomile Lightening Hydrogel Mask Pack [5pc</t>
+          <t>8809242276820</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>129</v>
-      </c>
-      <c r="E23" t="n">
-        <v>88</v>
-      </c>
+        <v>501</v>
+      </c>
+      <c r="E23" s="2" t="n"/>
       <c r="F23">
-        <f>E23*$J$3</f>
-        <v/>
-      </c>
-      <c r="G23">
-        <f>IF(F23=0,"",ROUND(D23/(F23/30),0))</f>
-        <v/>
-      </c>
-      <c r="H23">
-        <f>MAX(0,ROUND(F23*$J$2-D23,0))</f>
-        <v/>
-      </c>
-      <c r="I23">
-        <f>H23*$J$4/1000</f>
+        <f>D23*E23</f>
+        <v/>
+      </c>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23">
+        <f>IF(G23="","",ROUNDUP(D23/G23,0))</f>
+        <v/>
+      </c>
+      <c r="K23">
+        <f>IF(J23="","",J23*H23)</f>
+        <v/>
+      </c>
+      <c r="L23">
+        <f>IF(J23="","",J23*I23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EKEL</t>
+          <t>ROUND LAB</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>208202076</t>
+          <t>ROUND LAB SOYBEAN PANTHENOL CREAM_80ml - Крем для лица с чёр</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>EKEL - Ampule Сream Сollagen [70ml] / Крем для лица амп</t>
+          <t>8809875907337</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>324</v>
-      </c>
-      <c r="E24" t="n">
-        <v>83</v>
-      </c>
+        <v>406</v>
+      </c>
+      <c r="E24" s="2" t="n"/>
       <c r="F24">
-        <f>E24*$J$3</f>
-        <v/>
-      </c>
-      <c r="G24">
-        <f>IF(F24=0,"",ROUND(D24/(F24/30),0))</f>
-        <v/>
-      </c>
-      <c r="H24">
-        <f>MAX(0,ROUND(F24*$J$2-D24,0))</f>
-        <v/>
-      </c>
-      <c r="I24">
-        <f>H24*$J$4/1000</f>
+        <f>D24*E24</f>
+        <v/>
+      </c>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24">
+        <f>IF(G24="","",ROUNDUP(D24/G24,0))</f>
+        <v/>
+      </c>
+      <c r="K24">
+        <f>IF(J24="","",J24*H24)</f>
+        <v/>
+      </c>
+      <c r="L24">
+        <f>IF(J24="","",J24*I24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ROUND LAB</t>
+          <t>HEIMISH</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>437254254</t>
+          <t>HEIMISH - All Clean Balm Mandarin [120ml] / Очищающий гидроф</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROUND LAB SOYBEAN PANTHENOL CREAM_80ml - Крем для лица </t>
+          <t>8809481761996</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>310</v>
-      </c>
-      <c r="E25" t="n">
-        <v>72</v>
-      </c>
+        <v>562</v>
+      </c>
+      <c r="E25" s="2" t="n"/>
       <c r="F25">
-        <f>E25*$J$3</f>
-        <v/>
-      </c>
-      <c r="G25">
-        <f>IF(F25=0,"",ROUND(D25/(F25/30),0))</f>
-        <v/>
-      </c>
-      <c r="H25">
-        <f>MAX(0,ROUND(F25*$J$2-D25,0))</f>
-        <v/>
-      </c>
-      <c r="I25">
-        <f>H25*$J$4/1000</f>
+        <f>D25*E25</f>
+        <v/>
+      </c>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25">
+        <f>IF(G25="","",ROUNDUP(D25/G25,0))</f>
+        <v/>
+      </c>
+      <c r="K25">
+        <f>IF(J25="","",J25*H25)</f>
+        <v/>
+      </c>
+      <c r="L25">
+        <f>IF(J25="","",J25*I25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>HEIMISH</t>
+          <t>ETUDEHOUSE</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>207465786</t>
+          <t>ETUDE - Baking Powder Crunch Pore Scrub [24*7ml] / Очищающий</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>HEIMISH - All Clean Balm Mandarin [120ml] / Очищающий г</t>
+          <t>8809820692707</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>108</v>
-      </c>
-      <c r="E26" t="n">
-        <v>68</v>
-      </c>
+        <v>331</v>
+      </c>
+      <c r="E26" s="2" t="n"/>
       <c r="F26">
-        <f>E26*$J$3</f>
-        <v/>
-      </c>
-      <c r="G26">
-        <f>IF(F26=0,"",ROUND(D26/(F26/30),0))</f>
-        <v/>
-      </c>
-      <c r="H26">
-        <f>MAX(0,ROUND(F26*$J$2-D26,0))</f>
-        <v/>
-      </c>
-      <c r="I26">
-        <f>H26*$J$4/1000</f>
+        <f>D26*E26</f>
+        <v/>
+      </c>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="n"/>
+      <c r="J26">
+        <f>IF(G26="","",ROUNDUP(D26/G26,0))</f>
+        <v/>
+      </c>
+      <c r="K26">
+        <f>IF(J26="","",J26*H26)</f>
+        <v/>
+      </c>
+      <c r="L26">
+        <f>IF(J26="","",J26*I26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ETUDEHOUSE</t>
+          <t>PETITFEE</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>154160085</t>
+          <t xml:space="preserve">PETITFEE - Chamomile Lightening Hydrogel Eye Patch [60ea] / </t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ETUDE - Baking Powder Crunch Pore Scrub [24*7ml] / Очищ</t>
+          <t>8809508850412</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>309</v>
-      </c>
-      <c r="E27" t="n">
-        <v>65</v>
-      </c>
+        <v>138</v>
+      </c>
+      <c r="E27" s="2" t="n"/>
       <c r="F27">
-        <f>E27*$J$3</f>
-        <v/>
-      </c>
-      <c r="G27">
-        <f>IF(F27=0,"",ROUND(D27/(F27/30),0))</f>
-        <v/>
-      </c>
-      <c r="H27">
-        <f>MAX(0,ROUND(F27*$J$2-D27,0))</f>
-        <v/>
-      </c>
-      <c r="I27">
-        <f>H27*$J$4/1000</f>
+        <f>D27*E27</f>
+        <v/>
+      </c>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="2" t="n"/>
+      <c r="J27">
+        <f>IF(G27="","",ROUNDUP(D27/G27,0))</f>
+        <v/>
+      </c>
+      <c r="K27">
+        <f>IF(J27="","",J27*H27)</f>
+        <v/>
+      </c>
+      <c r="L27">
+        <f>IF(J27="","",J27*I27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PETITFEE</t>
+          <t>ETUDEHOUSE</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>179611318</t>
+          <t xml:space="preserve">ETUDE - Baking Powder BB Deep Cleansing Foam [30ml] / Пенка </t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PETITFEE - Chamomile Lightening Hydrogel Eye Patch [60e</t>
+          <t>8809668028058</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>357</v>
-      </c>
-      <c r="E28" t="n">
-        <v>50</v>
-      </c>
+        <v>317</v>
+      </c>
+      <c r="E28" s="2" t="n"/>
       <c r="F28">
-        <f>E28*$J$3</f>
-        <v/>
-      </c>
-      <c r="G28">
-        <f>IF(F28=0,"",ROUND(D28/(F28/30),0))</f>
-        <v/>
-      </c>
-      <c r="H28">
-        <f>MAX(0,ROUND(F28*$J$2-D28,0))</f>
-        <v/>
-      </c>
-      <c r="I28">
-        <f>H28*$J$4/1000</f>
+        <f>D28*E28</f>
+        <v/>
+      </c>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="n"/>
+      <c r="J28">
+        <f>IF(G28="","",ROUNDUP(D28/G28,0))</f>
+        <v/>
+      </c>
+      <c r="K28">
+        <f>IF(J28="","",J28*H28)</f>
+        <v/>
+      </c>
+      <c r="L28">
+        <f>IF(J28="","",J28*I28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ETUDEHOUSE</t>
+          <t>COSRX</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>154159632</t>
+          <t>COSRX - Advanced Snail 96 Mucin Power Essence [100ml] / Высо</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ETUDE - Baking Powder BB Deep Cleansing Foam [30ml] / П</t>
+          <t>8809416470009</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>175</v>
-      </c>
-      <c r="E29" t="n">
-        <v>50</v>
-      </c>
+        <v>414</v>
+      </c>
+      <c r="E29" s="2" t="n"/>
       <c r="F29">
-        <f>E29*$J$3</f>
-        <v/>
-      </c>
-      <c r="G29">
-        <f>IF(F29=0,"",ROUND(D29/(F29/30),0))</f>
-        <v/>
-      </c>
-      <c r="H29">
-        <f>MAX(0,ROUND(F29*$J$2-D29,0))</f>
-        <v/>
-      </c>
-      <c r="I29">
-        <f>H29*$J$4/1000</f>
+        <f>D29*E29</f>
+        <v/>
+      </c>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29">
+        <f>IF(G29="","",ROUNDUP(D29/G29,0))</f>
+        <v/>
+      </c>
+      <c r="K29">
+        <f>IF(J29="","",J29*H29)</f>
+        <v/>
+      </c>
+      <c r="L29">
+        <f>IF(J29="","",J29*I29)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>COSRX</t>
+          <t>ROUND LAB</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>207481251</t>
+          <t xml:space="preserve">ROUND LAB VITA NIACINAMIDE DARK SPOT SERUM 30ml - Сыворотка </t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>COSRX - Advanced Snail 96 Mucin Power Essence [100ml] /</t>
+          <t>8809962540652</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>38</v>
-      </c>
-      <c r="E30" t="n">
-        <v>46</v>
-      </c>
+        <v>337</v>
+      </c>
+      <c r="E30" s="2" t="n"/>
       <c r="F30">
-        <f>E30*$J$3</f>
-        <v/>
-      </c>
-      <c r="G30">
-        <f>IF(F30=0,"",ROUND(D30/(F30/30),0))</f>
-        <v/>
-      </c>
-      <c r="H30">
-        <f>MAX(0,ROUND(F30*$J$2-D30,0))</f>
-        <v/>
-      </c>
-      <c r="I30">
-        <f>H30*$J$4/1000</f>
+        <f>D30*E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30">
+        <f>IF(G30="","",ROUNDUP(D30/G30,0))</f>
+        <v/>
+      </c>
+      <c r="K30">
+        <f>IF(J30="","",J30*H30)</f>
+        <v/>
+      </c>
+      <c r="L30">
+        <f>IF(J30="","",J30*I30)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ROUND LAB</t>
+          <t>DEOPROCE</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>437797551</t>
+          <t>DEOPROCE SHAMPOO - BLACK GARLIC INTENSME ENERGY [600ml] мягк</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ROUND LAB VITA NIACINAMIDE DARK SPOT SERUM 30ml - Сывор</t>
+          <t>8809975191773</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>62</v>
-      </c>
-      <c r="E31" t="n">
-        <v>40</v>
-      </c>
+        <v>261</v>
+      </c>
+      <c r="E31" s="2" t="n"/>
       <c r="F31">
-        <f>E31*$J$3</f>
-        <v/>
-      </c>
-      <c r="G31">
-        <f>IF(F31=0,"",ROUND(D31/(F31/30),0))</f>
-        <v/>
-      </c>
-      <c r="H31">
-        <f>MAX(0,ROUND(F31*$J$2-D31,0))</f>
-        <v/>
-      </c>
-      <c r="I31">
-        <f>H31*$J$4/1000</f>
+        <f>D31*E31</f>
+        <v/>
+      </c>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31">
+        <f>IF(G31="","",ROUNDUP(D31/G31,0))</f>
+        <v/>
+      </c>
+      <c r="K31">
+        <f>IF(J31="","",J31*H31)</f>
+        <v/>
+      </c>
+      <c r="L31">
+        <f>IF(J31="","",J31*I31)</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DEOPROCE</t>
+          <t>ENOUGH</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>608837066</t>
+          <t xml:space="preserve">ENOUGH - Collagen Moisture Foundation [Tone 23] / Тональный </t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>DEOPROCE SHAMPOO - BLACK GARLIC INTENSME ENERGY [600ml]</t>
+          <t>8809280062386</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>122</v>
-      </c>
-      <c r="E32" t="n">
-        <v>39</v>
-      </c>
+        <v>243</v>
+      </c>
+      <c r="E32" s="2" t="n"/>
       <c r="F32">
-        <f>E32*$J$3</f>
-        <v/>
-      </c>
-      <c r="G32">
-        <f>IF(F32=0,"",ROUND(D32/(F32/30),0))</f>
-        <v/>
-      </c>
-      <c r="H32">
-        <f>MAX(0,ROUND(F32*$J$2-D32,0))</f>
-        <v/>
-      </c>
-      <c r="I32">
-        <f>H32*$J$4/1000</f>
+        <f>D32*E32</f>
+        <v/>
+      </c>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32">
+        <f>IF(G32="","",ROUNDUP(D32/G32,0))</f>
+        <v/>
+      </c>
+      <c r="K32">
+        <f>IF(J32="","",J32*H32)</f>
+        <v/>
+      </c>
+      <c r="L32">
+        <f>IF(J32="","",J32*I32)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ENOUGH</t>
+          <t>JIGOTT</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>611747838</t>
+          <t>JIGOTT - Collagen Healing Cream [100ml] / Крем для лица с ко</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ENOUGH - Collagen Moisture Foundation [Tone 23] / Тонал</t>
+          <t>8809210036524</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>90</v>
-      </c>
-      <c r="E33" t="n">
-        <v>34</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="E33" s="2" t="n"/>
       <c r="F33">
-        <f>E33*$J$3</f>
-        <v/>
-      </c>
-      <c r="G33">
-        <f>IF(F33=0,"",ROUND(D33/(F33/30),0))</f>
-        <v/>
-      </c>
-      <c r="H33">
-        <f>MAX(0,ROUND(F33*$J$2-D33,0))</f>
-        <v/>
-      </c>
-      <c r="I33">
-        <f>H33*$J$4/1000</f>
+        <f>D33*E33</f>
+        <v/>
+      </c>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33">
+        <f>IF(G33="","",ROUNDUP(D33/G33,0))</f>
+        <v/>
+      </c>
+      <c r="K33">
+        <f>IF(J33="","",J33*H33)</f>
+        <v/>
+      </c>
+      <c r="L33">
+        <f>IF(J33="","",J33*I33)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>JIGOTT</t>
+          <t>ROUND LAB</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>212753217</t>
+          <t>ROUND LAB PINE CALMING CICA AMPOULE_30ml - Сыворотка для жир</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>JIGOTT - Collagen Healing Cream [100ml] / Крем для лица</t>
+          <t>8809783325667</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>133</v>
-      </c>
-      <c r="E34" t="n">
-        <v>31</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="E34" s="2" t="n"/>
       <c r="F34">
-        <f>E34*$J$3</f>
-        <v/>
-      </c>
-      <c r="G34">
-        <f>IF(F34=0,"",ROUND(D34/(F34/30),0))</f>
-        <v/>
-      </c>
-      <c r="H34">
-        <f>MAX(0,ROUND(F34*$J$2-D34,0))</f>
-        <v/>
-      </c>
-      <c r="I34">
-        <f>H34*$J$4/1000</f>
+        <f>D34*E34</f>
+        <v/>
+      </c>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34">
+        <f>IF(G34="","",ROUNDUP(D34/G34,0))</f>
+        <v/>
+      </c>
+      <c r="K34">
+        <f>IF(J34="","",J34*H34)</f>
+        <v/>
+      </c>
+      <c r="L34">
+        <f>IF(J34="","",J34*I34)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ROUND LAB</t>
+          <t>DEOPROCE</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>437776835</t>
+          <t>DEOPROCE SHAMPOO - BLACK GARLIC INTENSME ENERGY [600ml] мягк</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ROUND LAB PINE CALMING CICA AMPOULE_30ml - Сыворотка дл</t>
+          <t>8809975191766</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>103</v>
-      </c>
-      <c r="E35" t="n">
-        <v>31</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="E35" s="2" t="n"/>
       <c r="F35">
-        <f>E35*$J$3</f>
-        <v/>
-      </c>
-      <c r="G35">
-        <f>IF(F35=0,"",ROUND(D35/(F35/30),0))</f>
-        <v/>
-      </c>
-      <c r="H35">
-        <f>MAX(0,ROUND(F35*$J$2-D35,0))</f>
-        <v/>
-      </c>
-      <c r="I35">
-        <f>H35*$J$4/1000</f>
+        <f>D35*E35</f>
+        <v/>
+      </c>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35">
+        <f>IF(G35="","",ROUNDUP(D35/G35,0))</f>
+        <v/>
+      </c>
+      <c r="K35">
+        <f>IF(J35="","",J35*H35)</f>
+        <v/>
+      </c>
+      <c r="L35">
+        <f>IF(J35="","",J35*I35)</f>
         <v/>
       </c>
     </row>
@@ -8791,360 +8864,320 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>608624295</t>
+          <t>DEOPROCE - SNAIL RECOVERY CREAM [100g] / Крем восстанавливаю</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>DEOPROCE SHAMPOO - BLACK GARLIC INTENSME ENERGY [600ml]</t>
+          <t>8809240760659</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>143</v>
-      </c>
-      <c r="E36" t="n">
-        <v>30</v>
-      </c>
+        <v>164</v>
+      </c>
+      <c r="E36" s="2" t="n"/>
       <c r="F36">
-        <f>E36*$J$3</f>
-        <v/>
-      </c>
-      <c r="G36">
-        <f>IF(F36=0,"",ROUND(D36/(F36/30),0))</f>
-        <v/>
-      </c>
-      <c r="H36">
-        <f>MAX(0,ROUND(F36*$J$2-D36,0))</f>
-        <v/>
-      </c>
-      <c r="I36">
-        <f>H36*$J$4/1000</f>
+        <f>D36*E36</f>
+        <v/>
+      </c>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36">
+        <f>IF(G36="","",ROUNDUP(D36/G36,0))</f>
+        <v/>
+      </c>
+      <c r="K36">
+        <f>IF(J36="","",J36*H36)</f>
+        <v/>
+      </c>
+      <c r="L36">
+        <f>IF(J36="","",J36*I36)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DEOPROCE</t>
+          <t>TheOrdinary</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>214304883</t>
+          <t>THE ORDINARY - Argireline Solution 10% [30ml] / Сыворотка дл</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>DEOPROCE - SNAIL RECOVERY CREAM [100g] / Крем восстанав</t>
+          <t>769915190946</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>57</v>
-      </c>
-      <c r="E37" t="n">
-        <v>22</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="E37" s="2" t="n"/>
       <c r="F37">
-        <f>E37*$J$3</f>
-        <v/>
-      </c>
-      <c r="G37">
-        <f>IF(F37=0,"",ROUND(D37/(F37/30),0))</f>
-        <v/>
-      </c>
-      <c r="H37">
-        <f>MAX(0,ROUND(F37*$J$2-D37,0))</f>
-        <v/>
-      </c>
-      <c r="I37">
-        <f>H37*$J$4/1000</f>
+        <f>D37*E37</f>
+        <v/>
+      </c>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37">
+        <f>IF(G37="","",ROUNDUP(D37/G37,0))</f>
+        <v/>
+      </c>
+      <c r="K37">
+        <f>IF(J37="","",J37*H37)</f>
+        <v/>
+      </c>
+      <c r="L37">
+        <f>IF(J37="","",J37*I37)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TheOrdinary</t>
+          <t>PETITFEE</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>214312385</t>
+          <t>PETITFEE - Aura Quartz Hydrogel Eye Patch [60ea]</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>THE ORDINARY - Argireline Solution 10% [30ml] / Сыворот</t>
+          <t>8809508850801</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>127</v>
-      </c>
-      <c r="E38" t="n">
-        <v>22</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="E38" s="2" t="n"/>
       <c r="F38">
-        <f>E38*$J$3</f>
-        <v/>
-      </c>
-      <c r="G38">
-        <f>IF(F38=0,"",ROUND(D38/(F38/30),0))</f>
-        <v/>
-      </c>
-      <c r="H38">
-        <f>MAX(0,ROUND(F38*$J$2-D38,0))</f>
-        <v/>
-      </c>
-      <c r="I38">
-        <f>H38*$J$4/1000</f>
+        <f>D38*E38</f>
+        <v/>
+      </c>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38">
+        <f>IF(G38="","",ROUNDUP(D38/G38,0))</f>
+        <v/>
+      </c>
+      <c r="K38">
+        <f>IF(J38="","",J38*H38)</f>
+        <v/>
+      </c>
+      <c r="L38">
+        <f>IF(J38="","",J38*I38)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PETITFEE</t>
+          <t>LEBELAGE</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>180992464</t>
+          <t xml:space="preserve">LEBELAGE - Dr. Hyaluronic Derma Eye Cream [40ml] / Крем для </t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PETITFEE - Aura Quartz Hydrogel Eye Patch [60ea]</t>
+          <t>8809445616522</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>126</v>
-      </c>
-      <c r="E39" t="n">
-        <v>20</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="E39" s="2" t="n"/>
       <c r="F39">
-        <f>E39*$J$3</f>
-        <v/>
-      </c>
-      <c r="G39">
-        <f>IF(F39=0,"",ROUND(D39/(F39/30),0))</f>
-        <v/>
-      </c>
-      <c r="H39">
-        <f>MAX(0,ROUND(F39*$J$2-D39,0))</f>
-        <v/>
-      </c>
-      <c r="I39">
-        <f>H39*$J$4/1000</f>
+        <f>D39*E39</f>
+        <v/>
+      </c>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39">
+        <f>IF(G39="","",ROUNDUP(D39/G39,0))</f>
+        <v/>
+      </c>
+      <c r="K39">
+        <f>IF(J39="","",J39*H39)</f>
+        <v/>
+      </c>
+      <c r="L39">
+        <f>IF(J39="","",J39*I39)</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LEBELAGE</t>
+          <t>ISNTREE</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>207818642</t>
+          <t>ISNTREE - Chestnut AHA 8% Clear Essence Sample [20ml] / Увла</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>LEBELAGE - Dr. Hyaluronic Derma Eye Cream [40ml] / Крем</t>
+          <t>8809088970357</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>39</v>
-      </c>
-      <c r="E40" t="n">
-        <v>19</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="E40" s="2" t="n"/>
       <c r="F40">
-        <f>E40*$J$3</f>
-        <v/>
-      </c>
-      <c r="G40">
-        <f>IF(F40=0,"",ROUND(D40/(F40/30),0))</f>
-        <v/>
-      </c>
-      <c r="H40">
-        <f>MAX(0,ROUND(F40*$J$2-D40,0))</f>
-        <v/>
-      </c>
-      <c r="I40">
-        <f>H40*$J$4/1000</f>
+        <f>D40*E40</f>
+        <v/>
+      </c>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40">
+        <f>IF(G40="","",ROUNDUP(D40/G40,0))</f>
+        <v/>
+      </c>
+      <c r="K40">
+        <f>IF(J40="","",J40*H40)</f>
+        <v/>
+      </c>
+      <c r="L40">
+        <f>IF(J40="","",J40*I40)</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ISNTREE</t>
+          <t>ROUND LAB</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>207818000</t>
+          <t>ROUND LAB SOYBEAN CLEANSING OIL_200ml - Гидрофильное масло д</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ISNTREE - Chestnut AHA 8% Clear Essence Sample [20ml] /</t>
+          <t>8809783322130</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>60</v>
-      </c>
-      <c r="E41" t="n">
-        <v>15</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="E41" s="2" t="n"/>
       <c r="F41">
-        <f>E41*$J$3</f>
-        <v/>
-      </c>
-      <c r="G41">
-        <f>IF(F41=0,"",ROUND(D41/(F41/30),0))</f>
-        <v/>
-      </c>
-      <c r="H41">
-        <f>MAX(0,ROUND(F41*$J$2-D41,0))</f>
-        <v/>
-      </c>
-      <c r="I41">
-        <f>H41*$J$4/1000</f>
+        <f>D41*E41</f>
+        <v/>
+      </c>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
+      <c r="I41" s="2" t="n"/>
+      <c r="J41">
+        <f>IF(G41="","",ROUNDUP(D41/G41,0))</f>
+        <v/>
+      </c>
+      <c r="K41">
+        <f>IF(J41="","",J41*H41)</f>
+        <v/>
+      </c>
+      <c r="L41">
+        <f>IF(J41="","",J41*I41)</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ROUND LAB</t>
+          <t>ENOUGH</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>437850261</t>
+          <t>ENOUGH Collagen whitening cover tip concealer #02 [9g]/Конси</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ROUND LAB SOYBEAN CLEANSING OIL_200ml - Гидрофильное ма</t>
+          <t>8809605872270</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>30</v>
-      </c>
-      <c r="E42" t="n">
-        <v>14</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="E42" s="2" t="n"/>
       <c r="F42">
-        <f>E42*$J$3</f>
-        <v/>
-      </c>
-      <c r="G42">
-        <f>IF(F42=0,"",ROUND(D42/(F42/30),0))</f>
-        <v/>
-      </c>
-      <c r="H42">
-        <f>MAX(0,ROUND(F42*$J$2-D42,0))</f>
-        <v/>
-      </c>
-      <c r="I42">
-        <f>H42*$J$4/1000</f>
+        <f>D42*E42</f>
+        <v/>
+      </c>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="n"/>
+      <c r="I42" s="2" t="n"/>
+      <c r="J42">
+        <f>IF(G42="","",ROUNDUP(D42/G42,0))</f>
+        <v/>
+      </c>
+      <c r="K42">
+        <f>IF(J42="","",J42*H42)</f>
+        <v/>
+      </c>
+      <c r="L42">
+        <f>IF(J42="","",J42*I42)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>ENOUGH</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>611744611</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>ENOUGH Collagen whitening cover tip concealer #02 [9g]/</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>5</v>
-      </c>
-      <c r="E43" t="n">
-        <v>8</v>
-      </c>
-      <c r="F43">
-        <f>E43*$J$3</f>
-        <v/>
-      </c>
-      <c r="G43">
-        <f>IF(F43=0,"",ROUND(D43/(F43/30),0))</f>
-        <v/>
-      </c>
-      <c r="H43">
-        <f>MAX(0,ROUND(F43*$J$2-D43,0))</f>
-        <v/>
-      </c>
-      <c r="I43">
-        <f>H43*$J$4/1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="C44" s="1" t="inlineStr">
+      <c r="B43" s="1" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="H44" s="1">
-        <f>SUM(H3:H43)</f>
-        <v/>
-      </c>
-      <c r="I44" s="1">
-        <f>SUM(I3:I43)</f>
+      <c r="D43" s="1">
+        <f>SUM(D2:D42)</f>
+        <v/>
+      </c>
+      <c r="F43" s="1">
+        <f>SUM(F2:F42)</f>
+        <v/>
+      </c>
+      <c r="K43" s="1">
+        <f>SUM(K2:K42)</f>
+        <v/>
+      </c>
+      <c r="L43" s="1">
+        <f>SUM(L2:L42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Вес контейнера, т</t>
+        </is>
+      </c>
+      <c r="D45">
+        <f>L43/1000</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Проверка веса, т</t>
-        </is>
-      </c>
-      <c r="D46">
-        <f>I44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Проверка штук</t>
-        </is>
-      </c>
-      <c r="D47">
-        <f>H44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>FarmStay исключён. Контейнер = позиции с покрытием &lt;150 дней, докуп до 6 мес спроса 2 магазинов.</t>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Лимит 26т/120к шт | транзит 2 мес | цель 6 мес | FarmStay искл. Жёлтые=ввод цены/короба (нет в заказе 22.06).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G3:G43">
-    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
-      <formula>90</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>